<commit_message>
log : Daily log of September 20.
</commit_message>
<xml_diff>
--- a/Development_DailyLog.xlsx
+++ b/Development_DailyLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\woo09\Desktop\DXlibrary\BloodEscape\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525D8950-679C-453E-A551-63F72B49F0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA67B29F-8105-4956-A836-60F6E78F9D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B4958722-2721-403E-AFBB-AC6F218FFB09}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>明日の予定</t>
     <rPh sb="0" eb="2">
@@ -109,6 +109,101 @@
     </rPh>
     <rPh sb="40" eb="42">
       <t>ジッソウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>プロジェクトのバージョン管理を行うリポジトリをGitHub上に作成した。
+また、テンプレートファイルを追加した。
+全てのステージからゲームオーバー画面に遷移できるように実装する必要がある。
+また、マップの実装の仕方も検討する必要がある。</t>
+    <rPh sb="12" eb="14">
+      <t>カンリ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>オコナ</t>
+    </rPh>
+    <rPh sb="29" eb="30">
+      <t>ジョウ</t>
+    </rPh>
+    <rPh sb="31" eb="33">
+      <t>サクセイ</t>
+    </rPh>
+    <rPh sb="51" eb="53">
+      <t>ツイカ</t>
+    </rPh>
+    <rPh sb="57" eb="58">
+      <t>スベ</t>
+    </rPh>
+    <rPh sb="73" eb="75">
+      <t>ガメン</t>
+    </rPh>
+    <rPh sb="76" eb="78">
+      <t>センイ</t>
+    </rPh>
+    <rPh sb="84" eb="86">
+      <t>ジッソウ</t>
+    </rPh>
+    <rPh sb="88" eb="90">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <rPh sb="102" eb="104">
+      <t>ジッソウ</t>
+    </rPh>
+    <rPh sb="105" eb="107">
+      <t>シカタ</t>
+    </rPh>
+    <rPh sb="108" eb="110">
+      <t>ケントウ</t>
+    </rPh>
+    <rPh sb="112" eb="114">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>午前:シーン管理の実装の仕方をChatGPTに聞く
+　　残りのテンプレートファイルの実装
+午後:素材の制作
+　　マップの実装の仕方をChatGPTに聞く</t>
+    <rPh sb="0" eb="2">
+      <t>ゴゼン</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>カンリ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ジッソウ</t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t>シカタ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="28" eb="29">
+      <t>ノコ</t>
+    </rPh>
+    <rPh sb="42" eb="44">
+      <t>ジッソウ</t>
+    </rPh>
+    <rPh sb="45" eb="47">
+      <t>ゴゴ</t>
+    </rPh>
+    <rPh sb="48" eb="50">
+      <t>ソザイ</t>
+    </rPh>
+    <rPh sb="51" eb="53">
+      <t>セイサク</t>
+    </rPh>
+    <rPh sb="60" eb="62">
+      <t>ジッソウ</t>
+    </rPh>
+    <rPh sb="63" eb="65">
+      <t>シカタ</t>
+    </rPh>
+    <rPh sb="74" eb="75">
+      <t>キ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -497,10 +592,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2888E61-A869-4B0D-9A7E-8B05AB5D3AE7}">
-  <dimension ref="B1:D2"/>
+  <dimension ref="B1:D3"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="3" max="3" width="59" customWidth="1"/>
+    <col min="3" max="3" width="70.1640625" customWidth="1"/>
     <col min="4" max="4" width="40.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -523,6 +618,17 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3" spans="2:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>